<commit_message>
data: drop 「（合成）」 from demo addresses
The header badge and help panel already say the data is fictional. Source,
bundled workbooks and archived samples patched in place (styles kept); a
snapshot saved with the old address still aligns to its footprint.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/demo/careflow-district-demo.xlsx
+++ b/public/demo/careflow-district-demo.xlsx
@@ -784,7 +784,7 @@
         <x:v>裕安樓</x:v>
       </x:c>
       <x:c r="C7" s="12" t="str">
-        <x:v>西營盤示範街 1 號（合成）</x:v>
+        <x:v>西營盤示範街 1 號</x:v>
       </x:c>
       <x:c r="D7" s="10" t="str">
         <x:v>1F：1F A室、1F B室、1F C室、1F D室
@@ -820,7 +820,7 @@
         <x:v>海景樓</x:v>
       </x:c>
       <x:c r="C8" s="13" t="str">
-        <x:v>西營盤示範街 8 號（合成）</x:v>
+        <x:v>西營盤示範街 8 號</x:v>
       </x:c>
       <x:c r="D8" s="11" t="str">
         <x:v>1F：1F A室、1F B室
@@ -850,7 +850,7 @@
         <x:v>德昌樓</x:v>
       </x:c>
       <x:c r="C9" s="12" t="str">
-        <x:v>西營盤示範街 16 號（合成）</x:v>
+        <x:v>西營盤示範街 16 號</x:v>
       </x:c>
       <x:c r="D9" s="10" t="str">
         <x:v>樓層／單位未核實</x:v>
@@ -879,7 +879,7 @@
         <x:v>安和樓</x:v>
       </x:c>
       <x:c r="C10" s="13" t="str">
-        <x:v>西營盤示範街 24 號（合成）</x:v>
+        <x:v>西營盤示範街 24 號</x:v>
       </x:c>
       <x:c r="D10" s="11" t="str">
         <x:v>樓層／單位未核實</x:v>
@@ -1560,7 +1560,7 @@
       </x:c>
       <x:c r="C7" s="18" t="str"/>
       <x:c r="D7" s="12" t="str">
-        <x:v>西營盤示範街 1 號（合成） 5F B室</x:v>
+        <x:v>西營盤示範街 1 號 5F B室</x:v>
       </x:c>
       <x:c r="E7" s="12" t="str"/>
       <x:c r="F7" s="10" t="str">
@@ -19221,7 +19221,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B7" s="37" t="str">
-        <x:v>{"schemaVersion":"0.1-demo","isSynthetic":true,"notice":"全區合成演示：20 個大廈位置用作介面測試；樓名、地址、樓層、單位、住戶及記錄均屬虛構，不代表地圖底圖中的真實建築或居民。依原紙本＋Excel 工作流設計，欄位仍待機構確認。","buildings":[{"isSynthetic":true,"provisional":true,"id":"bldg-yu-an","name":"裕安樓","address":"西營盤示範街 1 號（合成）","layoutDeclared":true,"floorCount":8,"initialCoverage":"UNVISITED","coordinates":{"lng":114.14178818464279,"lat":22.286363930711317},"footprint":[[114.14168894290924,22.286500432351488],[114.1418981552124,22.286495468660235],[114.14189279079437,22.286227429071147],[114.14167821407318,22.286237356472498],[114.14168894290924,22.286500432351488]]},{"isSynthetic":true,"provisional":true,"id":"bldg-hoi-king","name":"海景樓","address":"西營盤示範街 8 號（合成）","layoutDeclared":true,"floorCount":2,"initialCoverage":"UNVISITED","coordinates":{"lng":114.14255797863007,"lat":22.28661211534631},"footprint":[[114.14262235164642,22.286664234063778],[114.14262235164642,22.286619560888553],[114.14259016513824,22.286624524575387],[114.14258480072021,22.286589778763798],[114.14263308048248,22.286589778763798],[114.14263308048248,22.286555032943582],[114.14248287677765,22.286559996632704],[114.14248287677765,22.28659474245171],[114.14253115653992,22.28659474245171],[114.14253115653992,22.286624524575387],[114.14249897003174,22.286624524575387],[114.14249897003174,22.286669197749035],[114.14262235164642,22.286664234063778]]},{"isSynthetic":true,"provisional":true,"id":"bldg-duk-cheong","name":"德昌樓","address":"西營盤示範街 16 號（合成）","layoutDeclared":false,"initialCoverage":"UNKNOWN","coordinates":{"lng":114.14136976003647,"lat":22.286808180844794},"footprint":[[114.1414475440979,22.286733725641312],[114.14129197597504,22.286733725641312],[114.14129197597504,22.286882636048276],[114.1414475440979,22.286877672370593],[114.1414475440979,22.286733725641312]]},{"isSynthetic":true,"provisional":true,"id":"bldg-on-wo","name":"安和樓","address":"西營盤示範街 24 號（合成）","layoutDeclared":false,"initialCoverage":"UNKNOWN","coordinates":{"lng":114.14208590984344,"lat":22.28576580411479},"footprint":[[114.14213418960571,22.285825368723906],[114.14212882518768,22.28570127579063],[114.14203763008118,22.285706239510063],[114.1420429944992,22.285830332438948],[114.14213418960571,22.285825368723906]]},{"isSynthetic":true,"provisional":true,"id":"district-01","name":"晴里樓","address":"演示街區 01 號 · 虛構地址","coordinates":{"lng":114.13954049348831,"lat":22.287835658837054},"footprint":[[114.13945734500885,22.287890258967195],[114.13946807384491,22.287865440755937],[114.13947880268097,22.28787040439856],[114.13946270942688,22.287920040814882],[114.1395378112793,22.287939895376482],[114.13955390453339,22.287890258967195],[114.13956463336945,22.287890258967195],[114.13954854011536,22.287944859016434],[114.13962364196777,22.28796471357451],[114.13963973522186,22.287910113533016],[114.13965582847595,22.28791507717405],[114.13966655731201,22.28787536804097],[114.13965046405792,22.28787040439856],[114.13966119289398,22.287835658896626],[114.1396826505661,22.287840622540287],[114.13970410823822,22.28778105880474],[114.13943588733673,22.287706604099597],[114.1393768787384,22.28789522260891],[114.13945198059082,22.28791507717405],[114.13945734500885,22.287890258967195]],"layoutDeclared":true,"initialCoverage":"UNVISITED","floorCount":10},{"isSynthetic":true,"provisional":true,"id":"district-02","name":"青禾樓","address":"演示街區 02 號 · 虛構地址","coordinates":{"lng":114.14060264825821,"lat":22.287644558357755},"footprint":[[114.14048731327057,22.28780091338608],[114.14061069488525,22.28783069525278],[114.14062678813934,22.28778105880474],[114.1406911611557,22.287795949740996],[114.14071798324585,22.287696676802582],[114.14065897464752,22.28768178585574],[114.14071261882782,22.28749316705843],[114.1405838727951,22.28745842146273],[114.14048731327057,22.28780091338608]],"layoutDeclared":true,"initialCoverage":"UNVISITED","floorCount":7},{"isSynthetic":true,"provisional":true,"id":"district-03","name":"映榕樓","address":"演示街區 03 號 · 虛構地址","coordinates":{"lng":114.14200276136398,"lat":22.287753758732258},"footprint":[[114.14189279079437,22.287686749504857],[114.1418981552124,22.287825731608777],[114.1421127319336,22.28782076796459],[114.14210736751556,22.28768178585574],[114.14189279079437,22.287686749504857]],"layoutDeclared":true,"initialCoverage":"UNVISITED","floorCount":12},{"isSynthetic":true,"provisional":true,"id":"district-04","name":"小滿樓","address":"演示街區 04 號 · 虛構地址","coordinates":{"lng":114.14324462413788,"lat":22.287714049553372},"footprint":[[114.14331436157227,22.28778105880474],[114.14330899715424,22.28764207665641],[114.14319097995758,22.287647040306936],[114.14319097995758,22.287751276927438],[114.14317488670349,22.287751276927438],[114.14317488670349,22.287786022450334],[114.14331436157227,22.28778105880474]],"layoutDeclared":true,"initialCoverage":"UNVISITED","floorCount":5},{"isSynthetic":true,"provisional":true,"id":"district-05","name":"常悅樓","address":"演示街區 05 號 · 虛構地址","coordinates":{"lng":114.13936883211136,"lat":22.286842926596464},"footprint":[[114.13924276828766,22.28687270869274],[114.13945734500885,22.286927309139443],[114.13949489593506,22.286818108224736],[114.13928031921387,22.286758544053484],[114.13924276828766,22.28687270869274]],"layoutDeclared":true,"initialCoverage":"UNVISITED","floorCount":9},{"isSynthetic":true,"provisional":true,"id":"district-06","name":"知秋樓","address":"演示街區 06 號 · 虛構地址","coordinates":{"lng":114.14092719554901,"lat":22.286840444772693},"footprint":[[114.14082527160645,22.28683796294284],[114.14087355136871,22.28683796294284],[114.14087355136871,22.2868925634031],[114.14098620414734,22.286887599725773],[114.14098620414734,22.28683299926358],[114.14102911949158,22.28683299926358],[114.14102911949158,22.286788326142286],[114.14082527160645,22.286793289823123],[114.14082527160645,22.28683796294284]],"layoutDeclared":false,"initialCoverage":"UNVISITED"},{"isSynthetic":true,"provisional":true,"id":"district-07","name":"晴川樓","address":"演示街區 07 號 · 虛構地址","coordinates":{"lng":114.14216101169586,"lat":22.286723798239954},"footprint":[[114.14209127426147,22.286624524575387],[114.14209127426147,22.28665430669274],[114.14210200309753,22.28665430669274],[114.14210736751556,22.286793289823123],[114.1420966386795,22.286793289823123],[114.1420966386795,22.28682307190452],[114.14218246936798,22.28682307190452],[114.14217174053192,22.286763507735387],[114.14223074913025,22.286763507735387],[114.14223074913025,22.286674161434107],[114.14217174053192,22.286674161434107],[114.14217710494995,22.286624524575387],[114.14209127426147,22.286624524575387]],"layoutDeclared":true,"initialCoverage":"UNVISITED","floorCount":14},{"isSynthetic":true,"provisional":true,"id":"district-08","name":"穗安樓","address":"演示街區 08 號 · 虛構地址","coordinates":{"lng":114.14348870515823,"lat":22.286728761932885},"footprint":[[114.14357721805573,22.286644379321004],[114.14339482784271,22.286649343006957],[114.14340019226074,22.286813144544766],[114.14358258247375,22.286808180864625],[114.14357721805573,22.286644379321004]],"layoutDeclared":true,"initialCoverage":"UNVISITED","floorCount":6},{"isSynthetic":true,"provisional":true,"id":"district-09","name":"棠和樓","address":"演示街區 09 號 · 虛構地址","coordinates":{"lng":114.13955926895142,"lat":22.28589237884831},"footprint":[[114.13951098918915,22.28595442525767],[114.13961291313171,22.28594449783624],[114.13961291313171,22.28592960670275],[114.13965046405792,22.285924642991233],[114.13964509963989,22.285879969579653],[114.13960754871368,22.28588493329275],[114.13960218429565,22.285830332438948],[114.13955926895142,22.28583529615382],[114.13956463336945,22.285870042152922],[114.13954317569733,22.285870042152922],[114.13954317569733,22.28583529615382],[114.13950026035309,22.285840259868493],[114.13950562477112,22.285894860718443],[114.13946807384491,22.285894860718443],[114.13947343826294,22.285939534125234],[114.13951098918915,22.285939534125234],[114.13951098918915,22.28595442525767]],"layoutDeclared":true,"initialCoverage":"UNVISITED","floorCount":8},{"isSynthetic":true,"provisional":true,"id":"district-10","name":"日和樓","address":"演示街區 10 號 · 虛構地址","coordinates":{"lng":114.14058923721313,"lat":22.285837777977676},"footprint":[[114.1406375169754,22.285899824431013],[114.14064824581146,22.285899824431013],[114.14064288139343,22.28576580412968],[114.1406375169754,22.28576580412968],[114.14063215255737,22.285740985541267],[114.14057850837708,22.285745949259294],[114.14057850837708,22.285775731563803],[114.14056777954102,22.285775731563803],[114.14056241512299,22.285800550146064],[114.14053022861481,22.285800550146064],[114.14053022861481,22.285855151011503],[114.1405463218689,22.285855151011503],[114.1405463218689,22.285875005866373],[114.14053022861481,22.285875005866373],[114.14053559303284,22.285924642991233],[114.14062142372131,22.285934570414085],[114.14062142372131,22.28592960670275],[114.1406375169754,22.28592960670275],[114.1406375169754,22.285899824431013]],"layoutDeclared":true,"initialCoverage":"UNVISITED","floorCount":4},{"isSynthetic":true,"provisional":true,"id":"district-11","name":"朗月樓","address":"演示街區 11 號 · 虛構地址","coordinates":{"lng":114.14172112941742,"lat":22.285909751848486},"footprint":[[114.14187133312225,22.2858650784393],[114.14156556129456,22.285875005866373],[114.14156556129456,22.28595442525767],[114.14187669754028,22.28594449783624],[114.14187133312225,22.2858650784393]],"layoutDeclared":true,"initialCoverage":"UNVISITED","floorCount":11},{"isSynthetic":true,"provisional":true,"id":"district-12","name":"杏林樓","address":"演示街區 12 號 · 虛構地址","coordinates":{"lng":114.14298176765442,"lat":22.285726094375427},"footprint":[[114.14291203022003,22.28575091297715],[114.14291203022003,22.285780695280607],[114.14305686950684,22.285775731563803],[114.14305686950684,22.285671493470247],[114.142906665802,22.28567645719076],[114.14291203022003,22.28575091297715]],"layoutDeclared":false,"initialCoverage":"UNVISITED"},{"isSynthetic":true,"provisional":true,"id":"district-13","name":"拾光樓","address":"演示街區 13 號 · 虛構地址","coordinates":{"lng":114.13944393396378,"lat":22.284753202106018},"footprint":[[114.13941442966461,22.284693637093838],[114.13939833641052,22.284693637093838],[114.13935005664825,22.284668818315083],[114.13934469223022,22.284678745827122],[114.13930177688599,22.28465392704571],[114.13926959037781,22.2847184558682],[114.13938224315643,22.284768093403684],[114.13938760757446,22.284852477173544],[114.13942515850067,22.284847513423784],[114.13942515850067,22.284857440923133],[114.13946807384491,22.284857440923133],[114.13946270942688,22.284847513423784],[114.13950026035309,22.284842549673854],[114.13949489593506,22.284768093403684],[114.13961827754974,22.284698600849055],[114.13958609104156,22.2846489632889],[114.13954317569733,22.284668818315083],[114.1395378112793,22.284658890802348],[114.13947880268097,22.284688673338437],[114.13946270942688,22.284693637093838],[114.13946270942688,22.284673782071195],[114.13940906524658,22.284673782071195],[114.13941442966461,22.284693637093838]],"layoutDeclared":true,"initialCoverage":"UNVISITED","floorCount":13},{"isSynthetic":true,"provisional":true,"id":"district-14","name":"和煦樓","address":"演示街區 14 號 · 虛構地址","coordinates":{"lng":114.14081990718842,"lat":22.284790430151403},"footprint":[[114.14072871208191,22.284604289469698],[114.14073944091797,22.28498649835042],[114.14082527160645,22.284981534605436],[114.14082527160645,22.28496664336936],[114.14091110229492,22.28496664336936],[114.14090037345886,22.284594361952387],[114.14087355136871,22.284594361952387],[114.14087355136871,22.284604289469698],[114.14072871208191,22.284604289469698]],"layoutDeclared":true,"initialCoverage":"UNVISITED","floorCount":6},{"isSynthetic":true,"provisional":true,"id":"district-15","name":"榕溪樓","address":"演示街區 15 號 · 虛構地址","coordinates":{"lng":114.1420429944992,"lat":22.284894669027736},"footprint":[[114.14195716381073,22.284951752131732],[114.14212882518768,22.284946788385483],[114.14212346076965,22.28483758592374],[114.142005443573,22.28483758592374],[114.142005443573,22.284877295919713],[114.14195716381073,22.284882259668407],[114.14195716381073,22.284951752131732]],"layoutDeclared":true,"initialCoverage":"UNVISITED","floorCount":8},{"isSynthetic":true,"provisional":true,"id":"district-16","name":"微光樓","address":"演示街區 16 號 · 虛構地址","coordinates":{"lng":114.14333045482635,"lat":22.284941824574837},"footprint":[[114.14327681064606,22.285075845730304],[114.14339482784271,22.285070881988474],[114.14337873458862,22.28480780341937],[114.14326608181,22.284812767170536],[114.14327681064606,22.285075845730304]],"layoutDeclared":false,"initialCoverage":"UNKNOWN"}],"floors":[{"isSynthetic":true,"provisional":true,"id":"bldg-yu-an-f1","buildingId":"bldg-yu-an","label":"1F","level":1},{"isSynthetic":true,"provisional":true,"id":"bldg-yu-an-f2","buildingId":"bldg-yu-an","label":"2F","level":2},{"isSynthetic":true,"provisional":true,"id":"bldg-yu-an-f3","buildingId":"bldg-yu-an","label":"3F","level":3},{"isSynthetic":true,"provisional":true,"id":"bldg-yu-an-f4","buildingId":"bldg-yu-an","label":"4F","level":4},{"isSynthetic":true,"provisional":true,"id":"bldg-yu-an-f5","buildingId":"bldg-yu-an","label":"5F","level":5},{"isSynthetic":true,"provisional":true,"id":"bldg-yu-an-f6","buildingId":"bldg-yu-an","label":"6F","level":6},{"isSynthetic":true,"provisional":true,"id":"bldg-yu-an-f7","buildingId":"bldg-yu-an","label":"7F","level":7},{"isSynthetic":true,"provisional":true,"id":"bldg-yu-an-f8","buildingId":"bldg-yu-an","label":"8F","level":8},{"isSynthetic":true,"provisional":true,"id":"bldg-hoi-king-f1","buildingId":"bldg-hoi-king","label":"1F","level":1},{"isSynthetic":true,"provisional":true,"id":"bldg-hoi-king-f2","buildingId":"bldg-hoi-king","label":"2F","level":2},{"isSynthetic":true,"provisional":true,"id":"district-01-f1","buildingId":"district-01","level":1,"label":"1 樓"},{"isSynthetic":true,"provisional":true,"id":"district-01-f2","buildingId":"district-01","level":2,"label":"2 樓"},{"isSynthetic":true,"provisional":true,"id":"district-01-f3","buildingId":"district-01","level":3,"label":"3 樓"},{"isSynthetic":true,"provisional":true,"id":"district-01-f4","buildingId":"district-01","level":4,"label":"4 樓"},{"isSynthetic":true,"provisional":true,"id":"district-01-f5","buildingId":"district-01","level":5,"label":"5 樓"},{"isSynthetic":true,"provisional":true,"id":"district-01-f6","buildingId":"district-01","level":6,"label":"6 樓"},{"isSynthetic":true,"provisional":true,"id":"district-01-f7","buildingId":"district-01","level":7,"label":"7 樓"},{"isSynthetic":true,"provisional":true,"id":"district-01-f8","buildingId":"district-01","level":8,"label":"8 樓"},{"isSynthetic":true,"provisional":true,"id":"district-01-f9","buildingId":"district-01","level":9,"label":"9 樓"},{"isSynthetic":true,"provisional":true,"id":"district-01-f10","buildingId":"district-01","level":10,"label":"10 樓"},{"isSynthetic":true,"provisional":true,"id":"district-02-f1","buildingId":"district-02","level":1,"label":"1 樓"},{"isSynthetic":true,"provisional":true,"id":"district-02-f2","buildingId":"district-02","level":2,"label":"2 樓"},{"isSynthetic":true,"provisional":true,"id":"district-02-f3","buildingId":"district-02","level":3,"label":"3 樓"},{"isSynthetic":true,"provisional":true,"id":"district-02-f4","buildingId":"district-02","level":4,"label":"4 樓"},{"isSynthetic":true,"provisional":true,"id":"district-02-f5","buildingId":"district-02","level":5,"label":"5 樓"},{"isSynthetic":true,"provisional":true,"id":"district-02-f6","buildingId":"district-02","level":6,"label":"6 樓"},{"isSynthetic":true,"provisional":true,"id":"district-02-f7","buildingId":"district-02","level":7,"label":"7 樓"},{"isSynthetic":true,"provisional":true,"id":"district-03-f1","buildingId":"district-03","level":1,"label":"1 樓"},{"isSynthetic":true,"provisional":true,"id":"district-03-f2","buildingId":"district-03","level":2,"label":"2 樓"},{"isSynthetic":true,"provisional":true,"id":"district-03-f3","buildingId":"district-03","level":3,"label":"3 樓"},{"isSynthetic":true,"provisional":true,"id":"district-03-f4","buildingId":"district-03","level":4,"label":"4 樓"},{"isSynthetic":true,"provisional":true,"id":"district-03-f5","buildingId":"district-03","level":5,"label":"5 樓"},{"isSynthetic":true,"provisional":true,"id":"district-03-f6","buildingId":"district-03","level":6,"label":"6 樓"},{"isSynthetic":true,"provisional":true,"id":"district-03-f7","buildingId":"district-03","level":7,"label":"7 樓"},{"isSynthetic":true,"provisional":true,"id":"district-03-f8","buildingId":"district-03","level":8,"label":"8 樓"},{"isSynthetic":true,"provisional":true,"id":"district-03-f9","buildingId":"district-03","level":9,"label":"9 樓"},{"isSynthetic":true,"provisional":true,"id":"district-03-f10","buildingId":"district-03","level":10,"label":"10 樓"},{"isSynthetic":true,"provisional":true,"id":"district-03-f11","buildingId":"district-03","level":11,"label":"11 樓"},{"isSynthetic":true,"provisional":true,"id":"district-03-f12","buildingId":"district-03","level":12,"label":"12 樓"},{"isSynthetic":true,"provisional":true,"id":"district-04-f1","buildingId":"district-04","level":1,"label":"1 樓"},{"isSynthetic":true,"provisional":true,"id":"district-04-f2","buildingId":"district-04","level":2,"label":"2 樓"},{"isSynthetic":true,"provisional":true,"id":"district-04-f3","buildingId":"district-04","level":3,"label":"3 樓"},{"isSynthetic":true,"provisional":true,"id":"district-04-f4","buildingId":"district-04","level":4,"label":"4 樓"},{"isSynthetic":true,"provisional":true,"id":"district-04-f5","buildingId":"district-04","level":5,"label":"5 樓"},{"isSynthetic":true,"provisional":true,"id":"district-05-f1","buildingId":"district-05","level":1,"label":"1 樓"},{"isSynthetic":true,"provisional":true,"id":"district-05-f2","buildingId":"district-05","level":2,"label":"2 樓"},{"isSynthetic":true,"provisional":true,"id":"district-05-f3","buildingId":"district-05","level":3,"label":"3 樓"},{"isSynthetic":true,"provisional":true,"id":"district-05-f4","buildingId":"district-05","level":4,"label":"4 樓"},{"isSynthetic":true,"provisional":true,"id":"district-05-f5","buildingId":"district-05","level":5,"label":"5 樓"},{"isSynthetic":true,"provisional":true,"id":"district-05-f6","buildingId":"district-05","level":6,"label":"6 樓"},{"isSynthetic":true,"provisional":true,"id":"district-05-f7","buildingId":"district-05","level":7,"label":"7 樓"},{"isSynthetic":true,"provisional":true,"id":"district-05-f8","buildingId":"district-05","level":8,"label":"8 樓"},{"isSynthetic":true,"provisional":true,"id":"district-05-f9","buildingId":"district-05","level":9,"label":"9 樓"},{"isSynthetic":true,"provisional":true,"id":"district-07-f1","buildingId":"district-07","level":1,"label":"1 樓"},{"isSynthetic":true,"provisional":true,"id":"district-07-f2","buildingId":"district-07","level":2,"label":"2 樓"},{"isSynthetic":true,"provisional":true,"id":"district-07-f3","buildingId":"district-07","level":3,"label":"3 樓"},{"isSynthetic":true,"provisional":true,"id":"district-07-f4","buildingId":"district-07","level":4,"label":"4 樓"},{"isSynthetic":true,"provisional":true,"id":"district-07-f5","buildingId":"district-07","level":5,"label":"5 樓"},{"isSynthetic":true,"provisional":true,"id":"district-07-f6","buildingId":"district-07","level":6,"label":"6 樓"},{"isSynthetic":true,"provisional":true,"id":"district-07-f7","buildingId":"district-07","level":7,"label":"7 樓"},{"isSynthetic":true,"provisional":true,"id":"district-07-f8","buildingId":"district-07","level":8,"label":"8 樓"},{"isSynthetic":true,"provisional":true,"id":"district-07-f9","buildingId":"district-07","level":9,"label":"9 樓"},{"isSynthetic":true,"provisional":true,"id":"district-07-f10","buildingId":"district-07","level":10,"label":"10 樓"},{"isSynthetic":true,"provisional":true,"id":"district-07-f11","buildingId":"district-07","level":11,"label":"11 樓"},{"isSynthetic":true,"provisional":true,"id":"district-07-f12","buildingId":"district-07","level":12,"label":"12 樓"},{"isSynthetic":true,"provisional":true,"id":"district-07-f13","buildingId":"district-07","level":13,"label":"13 樓"},{"isSynthetic":true,"provisional":true,"id":"district-07-f14","buildingId":"district-07","level":14,"label":"14 樓"},{"isSynthetic":true,"provisional":true,"id":"district-08-f1","buildingId":"district-08","level":1,"label":"1 樓"},{"isSynthetic":true,"provisional":true,"id":"district-08-f2","buildingId":"district-08","level":2,"label":"2 樓"},{"isSynthetic":true,"provisional":true,"id":"district-08-f3","buildingId":"district-08","level":3,"label":"3 樓"},{"isSynthetic":true,"provisional":true,"id":"district-08-f4","buildingId":"district-08","level":4,"label":"4 樓"},{"isSynthetic":true,"provisional":true,"id":"district-08-f5","buildingId":"district-08","level":5,"label":"5 樓"},{"isSynthetic":true,"provisional":true,"id":"district-08-f6","buildingId":"district-08","level":6,"label":"6 樓"},{"isSynthetic":true,"provisional":true,"id":"district-09-f1","buildingId":"district-09","level":1,"label":"1 樓"},{"isSynthetic":true,"provisional":true,"id":"district-09-f2","buildingId":"district-09","level":2,"label":"2 樓"},{"isSynthetic":true,"provisional":true,"id":"district-09-f3","buildingId":"district-09","level":3,"label":"3 樓"},{"isSynthetic":true,"provisional":true,"id":"district-09-f4","buildingId":"district-09","level":4,"label":"4 樓"},{"isSynthetic":true,"provisional":true,"id":"district-09-f5","buildingId":"district-09","level":5,"label":"5 樓"},{"isSynthetic":true,"provisional":true,"id":"district-09-f6","buildingId":"district-09","level":6,"label":"6 樓"},{"isSynthetic":true,"provisional":true,"id":"district-09-f7","buildingId":"district-09","level":7,"label":"7 樓"},{"isSynthetic":true,"provisional":true,"id":"district-09-f8","buildingId":"district-09","level":8,"label":"8 樓"},{"isSynthetic":true,"provisional":true,"id":"district-10-f1","buildingId":"district-10","level":1,"label":"1 樓"},{"isSynthetic":true,"provisional":true,"id":"district-10-f2","buildingId":"district-10","level":2,"label":"2 樓"},{"isSynthetic":true,"provisional":true,"id":"district-10-f3","buildingId":"district-10","level":3,"label":"3 樓"},{"isSynthetic":true,"provisional":true,"id":"district-10-f4","buildingId":"district-10","level":4,"label":"4 樓"},{"isSynthetic":true,"provisional":true,"id":"district-11-f1","buildingId":"district-11","level":1,"label":"1 樓"},{"isSynthetic":true,"provisional":true,"id":"district-11-f2","buildingId":"district-11","level":2,"label":"2 樓"},{"isSynthetic":true,"provisional":true,"id":"district-11-f3","buildingId":"district-11","level":3,"label":"3 樓"},{"isSynthetic":true,"provisional":true,"id":"district-11-f4","buildingId":"district-11","level":4,"label":"4 樓"},{"isSynthetic":true,"provisional":true,"id":"district-11-f5","buildingId":"district-11","level":5,"label":"5 樓"},{"isSynthetic":true,"provisional":true,"id":"district-11-f6","buildingId":"district-11","level":6,"label":"6 樓"},{"isSynthetic":true,"provisional":true,"id":"district-11-f7","buildingId":"district-11","level":7,"label":"7 樓"},{"isSynthetic":true,"provisional":true,"id":"district-11-f8","buildingId":"district-11","level":8,"label":"8 樓"},{"isSynthetic":true,"provisional":true,"id":"district-11-f9","buildingId":"district-11","level":9,"label":"9 樓"},{"isSynthetic":true,"provisional":true,"id":"district-11-f10","buildingId":"district-11","level":10,"label":"10 樓"},{"isSynthetic":true,"provisional":true,"id":"district-11-f11","buildingId":"district-11","level":11,"label":"11 樓"},{"isSynthetic":true,"provisional":true,"id":"district-13-f1","buildingId":"district-13","level":1,"label":"1 樓"},{"isSynthetic":true,"provisional":true,"id":"district-13-f2","buildingId":"district-13","level":2,"label":"2 樓"},{"isSynthetic":true,"provisional":true,"id":"district-13-f3","buildingId":"district-13","level":3,"label":"3 樓"},{"isSynthetic":true,"provisional":true,"id":"district-13-f4","buildingId":"district-13","level":4,"label":"4 樓"},{"isSynthetic":true,"provisional":true,"id":"district-13-f5","buildingId":"district-13","level":5,"label":"5 樓"},{"isSynthetic":true,"provisional":true,"id":"district-13-f6","buildingId":"district-13","level":6,"label":"6 樓"},{"isSynthetic":true,"provisional":true,"id":"district-13-f7","buildingId":"district-13","level":7,"label":"7 樓"},{"isSynthetic":true,"provisional":true,"id":"district-13-f8","buildingId":"district-13","level":8,"label":"8 樓"},{"isSynthetic":true,"provisional":true,"id":"district-13-f9","buildingId":"district-13","level":9,"label":"9 樓"},{"isSynthetic":true,"provisional":true,"id":"district-13-f10","buildingId":"district-13","level":10,"label":"10 樓"},{"isSynthetic":true,"provisional":true,"id":"district-13-f11","buildingId":"district-13","level":11,"label":"11 樓"},{"isSynthetic":true,"provisional":true,"id":"district-13-f12","buildingId":"district-13","level":12,"label":"12 樓"},{"isSynthetic":true,"provisional":true,"id":"district-13-f13","buildingI</x:v>
+        <x:v>{"schemaVersion":"0.1-demo","isSynthetic":true,"notice":"全區合成演示：20 個大廈位置用作介面測試；樓名、地址、樓層、單位、住戶及記錄均屬虛構，不代表地圖底圖中的真實建築或居民。依原紙本＋Excel 工作流設計，欄位仍待機構確認。","buildings":[{"isSynthetic":true,"provisional":true,"id":"bldg-yu-an","name":"裕安樓","address":"西營盤示範街 1 號","layoutDeclared":true,"floorCount":8,"initialCoverage":"UNVISITED","coordinates":{"lng":114.14178818464279,"lat":22.286363930711317},"footprint":[[114.14168894290924,22.286500432351488],[114.1418981552124,22.286495468660235],[114.14189279079437,22.286227429071147],[114.14167821407318,22.286237356472498],[114.14168894290924,22.286500432351488]]},{"isSynthetic":true,"provisional":true,"id":"bldg-hoi-king","name":"海景樓","address":"西營盤示範街 8 號","layoutDeclared":true,"floorCount":2,"initialCoverage":"UNVISITED","coordinates":{"lng":114.14255797863007,"lat":22.28661211534631},"footprint":[[114.14262235164642,22.286664234063778],[114.14262235164642,22.286619560888553],[114.14259016513824,22.286624524575387],[114.14258480072021,22.286589778763798],[114.14263308048248,22.286589778763798],[114.14263308048248,22.286555032943582],[114.14248287677765,22.286559996632704],[114.14248287677765,22.28659474245171],[114.14253115653992,22.28659474245171],[114.14253115653992,22.286624524575387],[114.14249897003174,22.286624524575387],[114.14249897003174,22.286669197749035],[114.14262235164642,22.286664234063778]]},{"isSynthetic":true,"provisional":true,"id":"bldg-duk-cheong","name":"德昌樓","address":"西營盤示範街 16 號","layoutDeclared":false,"initialCoverage":"UNKNOWN","coordinates":{"lng":114.14136976003647,"lat":22.286808180844794},"footprint":[[114.1414475440979,22.286733725641312],[114.14129197597504,22.286733725641312],[114.14129197597504,22.286882636048276],[114.1414475440979,22.286877672370593],[114.1414475440979,22.286733725641312]]},{"isSynthetic":true,"provisional":true,"id":"bldg-on-wo","name":"安和樓","address":"西營盤示範街 24 號","layoutDeclared":false,"initialCoverage":"UNKNOWN","coordinates":{"lng":114.14208590984344,"lat":22.28576580411479},"footprint":[[114.14213418960571,22.285825368723906],[114.14212882518768,22.28570127579063],[114.14203763008118,22.285706239510063],[114.1420429944992,22.285830332438948],[114.14213418960571,22.285825368723906]]},{"isSynthetic":true,"provisional":true,"id":"district-01","name":"晴里樓","address":"演示街區 01 號 · 虛構地址","coordinates":{"lng":114.13954049348831,"lat":22.287835658837054},"footprint":[[114.13945734500885,22.287890258967195],[114.13946807384491,22.287865440755937],[114.13947880268097,22.28787040439856],[114.13946270942688,22.287920040814882],[114.1395378112793,22.287939895376482],[114.13955390453339,22.287890258967195],[114.13956463336945,22.287890258967195],[114.13954854011536,22.287944859016434],[114.13962364196777,22.28796471357451],[114.13963973522186,22.287910113533016],[114.13965582847595,22.28791507717405],[114.13966655731201,22.28787536804097],[114.13965046405792,22.28787040439856],[114.13966119289398,22.287835658896626],[114.1396826505661,22.287840622540287],[114.13970410823822,22.28778105880474],[114.13943588733673,22.287706604099597],[114.1393768787384,22.28789522260891],[114.13945198059082,22.28791507717405],[114.13945734500885,22.287890258967195]],"layoutDeclared":true,"initialCoverage":"UNVISITED","floorCount":10},{"isSynthetic":true,"provisional":true,"id":"district-02","name":"青禾樓","address":"演示街區 02 號 · 虛構地址","coordinates":{"lng":114.14060264825821,"lat":22.287644558357755},"footprint":[[114.14048731327057,22.28780091338608],[114.14061069488525,22.28783069525278],[114.14062678813934,22.28778105880474],[114.1406911611557,22.287795949740996],[114.14071798324585,22.287696676802582],[114.14065897464752,22.28768178585574],[114.14071261882782,22.28749316705843],[114.1405838727951,22.28745842146273],[114.14048731327057,22.28780091338608]],"layoutDeclared":true,"initialCoverage":"UNVISITED","floorCount":7},{"isSynthetic":true,"provisional":true,"id":"district-03","name":"映榕樓","address":"演示街區 03 號 · 虛構地址","coordinates":{"lng":114.14200276136398,"lat":22.287753758732258},"footprint":[[114.14189279079437,22.287686749504857],[114.1418981552124,22.287825731608777],[114.1421127319336,22.28782076796459],[114.14210736751556,22.28768178585574],[114.14189279079437,22.287686749504857]],"layoutDeclared":true,"initialCoverage":"UNVISITED","floorCount":12},{"isSynthetic":true,"provisional":true,"id":"district-04","name":"小滿樓","address":"演示街區 04 號 · 虛構地址","coordinates":{"lng":114.14324462413788,"lat":22.287714049553372},"footprint":[[114.14331436157227,22.28778105880474],[114.14330899715424,22.28764207665641],[114.14319097995758,22.287647040306936],[114.14319097995758,22.287751276927438],[114.14317488670349,22.287751276927438],[114.14317488670349,22.287786022450334],[114.14331436157227,22.28778105880474]],"layoutDeclared":true,"initialCoverage":"UNVISITED","floorCount":5},{"isSynthetic":true,"provisional":true,"id":"district-05","name":"常悅樓","address":"演示街區 05 號 · 虛構地址","coordinates":{"lng":114.13936883211136,"lat":22.286842926596464},"footprint":[[114.13924276828766,22.28687270869274],[114.13945734500885,22.286927309139443],[114.13949489593506,22.286818108224736],[114.13928031921387,22.286758544053484],[114.13924276828766,22.28687270869274]],"layoutDeclared":true,"initialCoverage":"UNVISITED","floorCount":9},{"isSynthetic":true,"provisional":true,"id":"district-06","name":"知秋樓","address":"演示街區 06 號 · 虛構地址","coordinates":{"lng":114.14092719554901,"lat":22.286840444772693},"footprint":[[114.14082527160645,22.28683796294284],[114.14087355136871,22.28683796294284],[114.14087355136871,22.2868925634031],[114.14098620414734,22.286887599725773],[114.14098620414734,22.28683299926358],[114.14102911949158,22.28683299926358],[114.14102911949158,22.286788326142286],[114.14082527160645,22.286793289823123],[114.14082527160645,22.28683796294284]],"layoutDeclared":false,"initialCoverage":"UNVISITED"},{"isSynthetic":true,"provisional":true,"id":"district-07","name":"晴川樓","address":"演示街區 07 號 · 虛構地址","coordinates":{"lng":114.14216101169586,"lat":22.286723798239954},"footprint":[[114.14209127426147,22.286624524575387],[114.14209127426147,22.28665430669274],[114.14210200309753,22.28665430669274],[114.14210736751556,22.286793289823123],[114.1420966386795,22.286793289823123],[114.1420966386795,22.28682307190452],[114.14218246936798,22.28682307190452],[114.14217174053192,22.286763507735387],[114.14223074913025,22.286763507735387],[114.14223074913025,22.286674161434107],[114.14217174053192,22.286674161434107],[114.14217710494995,22.286624524575387],[114.14209127426147,22.286624524575387]],"layoutDeclared":true,"initialCoverage":"UNVISITED","floorCount":14},{"isSynthetic":true,"provisional":true,"id":"district-08","name":"穗安樓","address":"演示街區 08 號 · 虛構地址","coordinates":{"lng":114.14348870515823,"lat":22.286728761932885},"footprint":[[114.14357721805573,22.286644379321004],[114.14339482784271,22.286649343006957],[114.14340019226074,22.286813144544766],[114.14358258247375,22.286808180864625],[114.14357721805573,22.286644379321004]],"layoutDeclared":true,"initialCoverage":"UNVISITED","floorCount":6},{"isSynthetic":true,"provisional":true,"id":"district-09","name":"棠和樓","address":"演示街區 09 號 · 虛構地址","coordinates":{"lng":114.13955926895142,"lat":22.28589237884831},"footprint":[[114.13951098918915,22.28595442525767],[114.13961291313171,22.28594449783624],[114.13961291313171,22.28592960670275],[114.13965046405792,22.285924642991233],[114.13964509963989,22.285879969579653],[114.13960754871368,22.28588493329275],[114.13960218429565,22.285830332438948],[114.13955926895142,22.28583529615382],[114.13956463336945,22.285870042152922],[114.13954317569733,22.285870042152922],[114.13954317569733,22.28583529615382],[114.13950026035309,22.285840259868493],[114.13950562477112,22.285894860718443],[114.13946807384491,22.285894860718443],[114.13947343826294,22.285939534125234],[114.13951098918915,22.285939534125234],[114.13951098918915,22.28595442525767]],"layoutDeclared":true,"initialCoverage":"UNVISITED","floorCount":8},{"isSynthetic":true,"provisional":true,"id":"district-10","name":"日和樓","address":"演示街區 10 號 · 虛構地址","coordinates":{"lng":114.14058923721313,"lat":22.285837777977676},"footprint":[[114.1406375169754,22.285899824431013],[114.14064824581146,22.285899824431013],[114.14064288139343,22.28576580412968],[114.1406375169754,22.28576580412968],[114.14063215255737,22.285740985541267],[114.14057850837708,22.285745949259294],[114.14057850837708,22.285775731563803],[114.14056777954102,22.285775731563803],[114.14056241512299,22.285800550146064],[114.14053022861481,22.285800550146064],[114.14053022861481,22.285855151011503],[114.1405463218689,22.285855151011503],[114.1405463218689,22.285875005866373],[114.14053022861481,22.285875005866373],[114.14053559303284,22.285924642991233],[114.14062142372131,22.285934570414085],[114.14062142372131,22.28592960670275],[114.1406375169754,22.28592960670275],[114.1406375169754,22.285899824431013]],"layoutDeclared":true,"initialCoverage":"UNVISITED","floorCount":4},{"isSynthetic":true,"provisional":true,"id":"district-11","name":"朗月樓","address":"演示街區 11 號 · 虛構地址","coordinates":{"lng":114.14172112941742,"lat":22.285909751848486},"footprint":[[114.14187133312225,22.2858650784393],[114.14156556129456,22.285875005866373],[114.14156556129456,22.28595442525767],[114.14187669754028,22.28594449783624],[114.14187133312225,22.2858650784393]],"layoutDeclared":true,"initialCoverage":"UNVISITED","floorCount":11},{"isSynthetic":true,"provisional":true,"id":"district-12","name":"杏林樓","address":"演示街區 12 號 · 虛構地址","coordinates":{"lng":114.14298176765442,"lat":22.285726094375427},"footprint":[[114.14291203022003,22.28575091297715],[114.14291203022003,22.285780695280607],[114.14305686950684,22.285775731563803],[114.14305686950684,22.285671493470247],[114.142906665802,22.28567645719076],[114.14291203022003,22.28575091297715]],"layoutDeclared":false,"initialCoverage":"UNVISITED"},{"isSynthetic":true,"provisional":true,"id":"district-13","name":"拾光樓","address":"演示街區 13 號 · 虛構地址","coordinates":{"lng":114.13944393396378,"lat":22.284753202106018},"footprint":[[114.13941442966461,22.284693637093838],[114.13939833641052,22.284693637093838],[114.13935005664825,22.284668818315083],[114.13934469223022,22.284678745827122],[114.13930177688599,22.28465392704571],[114.13926959037781,22.2847184558682],[114.13938224315643,22.284768093403684],[114.13938760757446,22.284852477173544],[114.13942515850067,22.284847513423784],[114.13942515850067,22.284857440923133],[114.13946807384491,22.284857440923133],[114.13946270942688,22.284847513423784],[114.13950026035309,22.284842549673854],[114.13949489593506,22.284768093403684],[114.13961827754974,22.284698600849055],[114.13958609104156,22.2846489632889],[114.13954317569733,22.284668818315083],[114.1395378112793,22.284658890802348],[114.13947880268097,22.284688673338437],[114.13946270942688,22.284693637093838],[114.13946270942688,22.284673782071195],[114.13940906524658,22.284673782071195],[114.13941442966461,22.284693637093838]],"layoutDeclared":true,"initialCoverage":"UNVISITED","floorCount":13},{"isSynthetic":true,"provisional":true,"id":"district-14","name":"和煦樓","address":"演示街區 14 號 · 虛構地址","coordinates":{"lng":114.14081990718842,"lat":22.284790430151403},"footprint":[[114.14072871208191,22.284604289469698],[114.14073944091797,22.28498649835042],[114.14082527160645,22.284981534605436],[114.14082527160645,22.28496664336936],[114.14091110229492,22.28496664336936],[114.14090037345886,22.284594361952387],[114.14087355136871,22.284594361952387],[114.14087355136871,22.284604289469698],[114.14072871208191,22.284604289469698]],"layoutDeclared":true,"initialCoverage":"UNVISITED","floorCount":6},{"isSynthetic":true,"provisional":true,"id":"district-15","name":"榕溪樓","address":"演示街區 15 號 · 虛構地址","coordinates":{"lng":114.1420429944992,"lat":22.284894669027736},"footprint":[[114.14195716381073,22.284951752131732],[114.14212882518768,22.284946788385483],[114.14212346076965,22.28483758592374],[114.142005443573,22.28483758592374],[114.142005443573,22.284877295919713],[114.14195716381073,22.284882259668407],[114.14195716381073,22.284951752131732]],"layoutDeclared":true,"initialCoverage":"UNVISITED","floorCount":8},{"isSynthetic":true,"provisional":true,"id":"district-16","name":"微光樓","address":"演示街區 16 號 · 虛構地址","coordinates":{"lng":114.14333045482635,"lat":22.284941824574837},"footprint":[[114.14327681064606,22.285075845730304],[114.14339482784271,22.285070881988474],[114.14337873458862,22.28480780341937],[114.14326608181,22.284812767170536],[114.14327681064606,22.285075845730304]],"layoutDeclared":false,"initialCoverage":"UNKNOWN"}],"floors":[{"isSynthetic":true,"provisional":true,"id":"bldg-yu-an-f1","buildingId":"bldg-yu-an","label":"1F","level":1},{"isSynthetic":true,"provisional":true,"id":"bldg-yu-an-f2","buildingId":"bldg-yu-an","label":"2F","level":2},{"isSynthetic":true,"provisional":true,"id":"bldg-yu-an-f3","buildingId":"bldg-yu-an","label":"3F","level":3},{"isSynthetic":true,"provisional":true,"id":"bldg-yu-an-f4","buildingId":"bldg-yu-an","label":"4F","level":4},{"isSynthetic":true,"provisional":true,"id":"bldg-yu-an-f5","buildingId":"bldg-yu-an","label":"5F","level":5},{"isSynthetic":true,"provisional":true,"id":"bldg-yu-an-f6","buildingId":"bldg-yu-an","label":"6F","level":6},{"isSynthetic":true,"provisional":true,"id":"bldg-yu-an-f7","buildingId":"bldg-yu-an","label":"7F","level":7},{"isSynthetic":true,"provisional":true,"id":"bldg-yu-an-f8","buildingId":"bldg-yu-an","label":"8F","level":8},{"isSynthetic":true,"provisional":true,"id":"bldg-hoi-king-f1","buildingId":"bldg-hoi-king","label":"1F","level":1},{"isSynthetic":true,"provisional":true,"id":"bldg-hoi-king-f2","buildingId":"bldg-hoi-king","label":"2F","level":2},{"isSynthetic":true,"provisional":true,"id":"district-01-f1","buildingId":"district-01","level":1,"label":"1 樓"},{"isSynthetic":true,"provisional":true,"id":"district-01-f2","buildingId":"district-01","level":2,"label":"2 樓"},{"isSynthetic":true,"provisional":true,"id":"district-01-f3","buildingId":"district-01","level":3,"label":"3 樓"},{"isSynthetic":true,"provisional":true,"id":"district-01-f4","buildingId":"district-01","level":4,"label":"4 樓"},{"isSynthetic":true,"provisional":true,"id":"district-01-f5","buildingId":"district-01","level":5,"label":"5 樓"},{"isSynthetic":true,"provisional":true,"id":"district-01-f6","buildingId":"district-01","level":6,"label":"6 樓"},{"isSynthetic":true,"provisional":true,"id":"district-01-f7","buildingId":"district-01","level":7,"label":"7 樓"},{"isSynthetic":true,"provisional":true,"id":"district-01-f8","buildingId":"district-01","level":8,"label":"8 樓"},{"isSynthetic":true,"provisional":true,"id":"district-01-f9","buildingId":"district-01","level":9,"label":"9 樓"},{"isSynthetic":true,"provisional":true,"id":"district-01-f10","buildingId":"district-01","level":10,"label":"10 樓"},{"isSynthetic":true,"provisional":true,"id":"district-02-f1","buildingId":"district-02","level":1,"label":"1 樓"},{"isSynthetic":true,"provisional":true,"id":"district-02-f2","buildingId":"district-02","level":2,"label":"2 樓"},{"isSynthetic":true,"provisional":true,"id":"district-02-f3","buildingId":"district-02","level":3,"label":"3 樓"},{"isSynthetic":true,"provisional":true,"id":"district-02-f4","buildingId":"district-02","level":4,"label":"4 樓"},{"isSynthetic":true,"provisional":true,"id":"district-02-f5","buildingId":"district-02","level":5,"label":"5 樓"},{"isSynthetic":true,"provisional":true,"id":"district-02-f6","buildingId":"district-02","level":6,"label":"6 樓"},{"isSynthetic":true,"provisional":true,"id":"district-02-f7","buildingId":"district-02","level":7,"label":"7 樓"},{"isSynthetic":true,"provisional":true,"id":"district-03-f1","buildingId":"district-03","level":1,"label":"1 樓"},{"isSynthetic":true,"provisional":true,"id":"district-03-f2","buildingId":"district-03","level":2,"label":"2 樓"},{"isSynthetic":true,"provisional":true,"id":"district-03-f3","buildingId":"district-03","level":3,"label":"3 樓"},{"isSynthetic":true,"provisional":true,"id":"district-03-f4","buildingId":"district-03","level":4,"label":"4 樓"},{"isSynthetic":true,"provisional":true,"id":"district-03-f5","buildingId":"district-03","level":5,"label":"5 樓"},{"isSynthetic":true,"provisional":true,"id":"district-03-f6","buildingId":"district-03","level":6,"label":"6 樓"},{"isSynthetic":true,"provisional":true,"id":"district-03-f7","buildingId":"district-03","level":7,"label":"7 樓"},{"isSynthetic":true,"provisional":true,"id":"district-03-f8","buildingId":"district-03","level":8,"label":"8 樓"},{"isSynthetic":true,"provisional":true,"id":"district-03-f9","buildingId":"district-03","level":9,"label":"9 樓"},{"isSynthetic":true,"provisional":true,"id":"district-03-f10","buildingId":"district-03","level":10,"label":"10 樓"},{"isSynthetic":true,"provisional":true,"id":"district-03-f11","buildingId":"district-03","level":11,"label":"11 樓"},{"isSynthetic":true,"provisional":true,"id":"district-03-f12","buildingId":"district-03","level":12,"label":"12 樓"},{"isSynthetic":true,"provisional":true,"id":"district-04-f1","buildingId":"district-04","level":1,"label":"1 樓"},{"isSynthetic":true,"provisional":true,"id":"district-04-f2","buildingId":"district-04","level":2,"label":"2 樓"},{"isSynthetic":true,"provisional":true,"id":"district-04-f3","buildingId":"district-04","level":3,"label":"3 樓"},{"isSynthetic":true,"provisional":true,"id":"district-04-f4","buildingId":"district-04","level":4,"label":"4 樓"},{"isSynthetic":true,"provisional":true,"id":"district-04-f5","buildingId":"district-04","level":5,"label":"5 樓"},{"isSynthetic":true,"provisional":true,"id":"district-05-f1","buildingId":"district-05","level":1,"label":"1 樓"},{"isSynthetic":true,"provisional":true,"id":"district-05-f2","buildingId":"district-05","level":2,"label":"2 樓"},{"isSynthetic":true,"provisional":true,"id":"district-05-f3","buildingId":"district-05","level":3,"label":"3 樓"},{"isSynthetic":true,"provisional":true,"id":"district-05-f4","buildingId":"district-05","level":4,"label":"4 樓"},{"isSynthetic":true,"provisional":true,"id":"district-05-f5","buildingId":"district-05","level":5,"label":"5 樓"},{"isSynthetic":true,"provisional":true,"id":"district-05-f6","buildingId":"district-05","level":6,"label":"6 樓"},{"isSynthetic":true,"provisional":true,"id":"district-05-f7","buildingId":"district-05","level":7,"label":"7 樓"},{"isSynthetic":true,"provisional":true,"id":"district-05-f8","buildingId":"district-05","level":8,"label":"8 樓"},{"isSynthetic":true,"provisional":true,"id":"district-05-f9","buildingId":"district-05","level":9,"label":"9 樓"},{"isSynthetic":true,"provisional":true,"id":"district-07-f1","buildingId":"district-07","level":1,"label":"1 樓"},{"isSynthetic":true,"provisional":true,"id":"district-07-f2","buildingId":"district-07","level":2,"label":"2 樓"},{"isSynthetic":true,"provisional":true,"id":"district-07-f3","buildingId":"district-07","level":3,"label":"3 樓"},{"isSynthetic":true,"provisional":true,"id":"district-07-f4","buildingId":"district-07","level":4,"label":"4 樓"},{"isSynthetic":true,"provisional":true,"id":"district-07-f5","buildingId":"district-07","level":5,"label":"5 樓"},{"isSynthetic":true,"provisional":true,"id":"district-07-f6","buildingId":"district-07","level":6,"label":"6 樓"},{"isSynthetic":true,"provisional":true,"id":"district-07-f7","buildingId":"district-07","level":7,"label":"7 樓"},{"isSynthetic":true,"provisional":true,"id":"district-07-f8","buildingId":"district-07","level":8,"label":"8 樓"},{"isSynthetic":true,"provisional":true,"id":"district-07-f9","buildingId":"district-07","level":9,"label":"9 樓"},{"isSynthetic":true,"provisional":true,"id":"district-07-f10","buildingId":"district-07","level":10,"label":"10 樓"},{"isSynthetic":true,"provisional":true,"id":"district-07-f11","buildingId":"district-07","level":11,"label":"11 樓"},{"isSynthetic":true,"provisional":true,"id":"district-07-f12","buildingId":"district-07","level":12,"label":"12 樓"},{"isSynthetic":true,"provisional":true,"id":"district-07-f13","buildingId":"district-07","level":13,"label":"13 樓"},{"isSynthetic":true,"provisional":true,"id":"district-07-f14","buildingId":"district-07","level":14,"label":"14 樓"},{"isSynthetic":true,"provisional":true,"id":"district-08-f1","buildingId":"district-08","level":1,"label":"1 樓"},{"isSynthetic":true,"provisional":true,"id":"district-08-f2","buildingId":"district-08","level":2,"label":"2 樓"},{"isSynthetic":true,"provisional":true,"id":"district-08-f3","buildingId":"district-08","level":3,"label":"3 樓"},{"isSynthetic":true,"provisional":true,"id":"district-08-f4","buildingId":"district-08","level":4,"label":"4 樓"},{"isSynthetic":true,"provisional":true,"id":"district-08-f5","buildingId":"district-08","level":5,"label":"5 樓"},{"isSynthetic":true,"provisional":true,"id":"district-08-f6","buildingId":"district-08","level":6,"label":"6 樓"},{"isSynthetic":true,"provisional":true,"id":"district-09-f1","buildingId":"district-09","level":1,"label":"1 樓"},{"isSynthetic":true,"provisional":true,"id":"district-09-f2","buildingId":"district-09","level":2,"label":"2 樓"},{"isSynthetic":true,"provisional":true,"id":"district-09-f3","buildingId":"district-09","level":3,"label":"3 樓"},{"isSynthetic":true,"provisional":true,"id":"district-09-f4","buildingId":"district-09","level":4,"label":"4 樓"},{"isSynthetic":true,"provisional":true,"id":"district-09-f5","buildingId":"district-09","level":5,"label":"5 樓"},{"isSynthetic":true,"provisional":true,"id":"district-09-f6","buildingId":"district-09","level":6,"label":"6 樓"},{"isSynthetic":true,"provisional":true,"id":"district-09-f7","buildingId":"district-09","level":7,"label":"7 樓"},{"isSynthetic":true,"provisional":true,"id":"district-09-f8","buildingId":"district-09","level":8,"label":"8 樓"},{"isSynthetic":true,"provisional":true,"id":"district-10-f1","buildingId":"district-10","level":1,"label":"1 樓"},{"isSynthetic":true,"provisional":true,"id":"district-10-f2","buildingId":"district-10","level":2,"label":"2 樓"},{"isSynthetic":true,"provisional":true,"id":"district-10-f3","buildingId":"district-10","level":3,"label":"3 樓"},{"isSynthetic":true,"provisional":true,"id":"district-10-f4","buildingId":"district-10","level":4,"label":"4 樓"},{"isSynthetic":true,"provisional":true,"id":"district-11-f1","buildingId":"district-11","level":1,"label":"1 樓"},{"isSynthetic":true,"provisional":true,"id":"district-11-f2","buildingId":"district-11","level":2,"label":"2 樓"},{"isSynthetic":true,"provisional":true,"id":"district-11-f3","buildingId":"district-11","level":3,"label":"3 樓"},{"isSynthetic":true,"provisional":true,"id":"district-11-f4","buildingId":"district-11","level":4,"label":"4 樓"},{"isSynthetic":true,"provisional":true,"id":"district-11-f5","buildingId":"district-11","level":5,"label":"5 樓"},{"isSynthetic":true,"provisional":true,"id":"district-11-f6","buildingId":"district-11","level":6,"label":"6 樓"},{"isSynthetic":true,"provisional":true,"id":"district-11-f7","buildingId":"district-11","level":7,"label":"7 樓"},{"isSynthetic":true,"provisional":true,"id":"district-11-f8","buildingId":"district-11","level":8,"label":"8 樓"},{"isSynthetic":true,"provisional":true,"id":"district-11-f9","buildingId":"district-11","level":9,"label":"9 樓"},{"isSynthetic":true,"provisional":true,"id":"district-11-f10","buildingId":"district-11","level":10,"label":"10 樓"},{"isSynthetic":true,"provisional":true,"id":"district-11-f11","buildingId":"district-11","level":11,"label":"11 樓"},{"isSynthetic":true,"provisional":true,"id":"district-13-f1","buildingId":"district-13","level":1,"label":"1 樓"},{"isSynthetic":true,"provisional":true,"id":"district-13-f2","buildingId":"district-13","level":2,"label":"2 樓"},{"isSynthetic":true,"provisional":true,"id":"district-13-f3","buildingId":"district-13","level":3,"label":"3 樓"},{"isSynthetic":true,"provisional":true,"id":"district-13-f4","buildingId":"district-13","level":4,"label":"4 樓"},{"isSynthetic":true,"provisional":true,"id":"district-13-f5","buildingId":"district-13","level":5,"label":"5 樓"},{"isSynthetic":true,"provisional":true,"id":"district-13-f6","buildingId":"district-13","level":6,"label":"6 樓"},{"isSynthetic":true,"provisional":true,"id":"district-13-f7","buildingId":"district-13","level":7,"label":"7 樓"},{"isSynthetic":true,"provisional":true,"id":"district-13-f8","buildingId":"district-13","level":8,"label":"8 樓"},{"isSynthetic":true,"provisional":true,"id":"district-13-f9","buildingId":"district-13","level":9,"label":"9 樓"},{"isSynthetic":true,"provisional":true,"id":"district-13-f10","buildingId":"district-13","level":10,"label":"10 樓"},{"isSynthetic":true,"provisional":true,"id":"district-13-f11","buildingId":"district-13","level":11,"label":"11 樓"},{"isSynthetic":true,"provisional":true,"id":"district-13-f12","buildingId":"district-13","level":12,"label":"12 樓"},{"isSynthetic":true,"provisional":true,"id":"district-13-f13","buildingI</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="25" customHeight="1">

</xml_diff>